<commit_message>
Update machine learning dataset and Apriori rules with latest data
</commit_message>
<xml_diff>
--- a/data/Rekomendasi_CrossSell.xlsx
+++ b/data/Rekomendasi_CrossSell.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O11"/>
+  <dimension ref="A1:O13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -508,530 +508,636 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>frozenset({'Lemon Tea Ice'})</t>
+          <t>frozenset({'Cappucino Hot Light'})</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>frozenset({'Nasi Goreng Sambal Ijo'})</t>
+          <t>frozenset({'Latte Ice Bold'})</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>0.01338055883510429</v>
+        <v>0.01309038284436258</v>
       </c>
       <c r="D2" t="n">
-        <v>0.02397051983828843</v>
+        <v>0.04604657281936587</v>
       </c>
       <c r="E2" t="n">
-        <v>0.00128796823011699</v>
+        <v>0.001184054729640837</v>
       </c>
       <c r="F2" t="n">
-        <v>0.09625668449197859</v>
+        <v>0.09045226130653267</v>
       </c>
       <c r="G2" t="n">
-        <v>4.015627743634766</v>
+        <v>1.964364680545585</v>
       </c>
       <c r="H2" t="n">
         <v>1</v>
       </c>
       <c r="I2" t="n">
-        <v>0.0009672292791127374</v>
+        <v>0.0005812874627645173</v>
       </c>
       <c r="J2" t="n">
-        <v>1.079985282782485</v>
+        <v>1.048821723806332</v>
       </c>
       <c r="K2" t="n">
-        <v>0.7611576474759562</v>
+        <v>0.4974412524902427</v>
       </c>
       <c r="L2" t="n">
-        <v>0.03571428571428571</v>
+        <v>0.02043132803632236</v>
       </c>
       <c r="M2" t="n">
-        <v>0.0740614562602285</v>
+        <v>0.04654911573451314</v>
       </c>
       <c r="N2" t="n">
-        <v>0.07499401388778033</v>
+        <v>0.05808327351040919</v>
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>frozenset({'Lemon Tea Ice', 'Nasi Goreng Sambal Ijo'})</t>
+          <t>frozenset({'Cappucino Hot Light', 'Latte Ice Bold'})</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>frozenset({'Iced Lychee Tea'})</t>
+          <t>frozenset({'Americano Hot Bold'})</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>frozenset({'Nasi Goreng Sambal Ijo'})</t>
+          <t>frozenset({'Americano Ice Bold'})</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>0.01749490179242245</v>
+        <v>0.01795816339955269</v>
       </c>
       <c r="D3" t="n">
-        <v>0.02397051983828843</v>
+        <v>0.06268911985265097</v>
       </c>
       <c r="E3" t="n">
-        <v>0.001431075811241101</v>
+        <v>0.001644520457834495</v>
       </c>
       <c r="F3" t="n">
-        <v>0.08179959100204499</v>
+        <v>0.09157509157509158</v>
       </c>
       <c r="G3" t="n">
-        <v>3.412508012086805</v>
+        <v>1.460781261410852</v>
       </c>
       <c r="H3" t="n">
         <v>1</v>
       </c>
       <c r="I3" t="n">
-        <v>0.00101171392075693</v>
+        <v>0.0005187390001464469</v>
       </c>
       <c r="J3" t="n">
-        <v>1.062980881512421</v>
+        <v>1.031797864033171</v>
       </c>
       <c r="K3" t="n">
-        <v>0.719548831112082</v>
+        <v>0.3212030276642776</v>
       </c>
       <c r="L3" t="n">
-        <v>0.03574620196604111</v>
+        <v>0.02081598667776852</v>
       </c>
       <c r="M3" t="n">
-        <v>0.05924930787354421</v>
+        <v>0.03081792000312599</v>
       </c>
       <c r="N3" t="n">
-        <v>0.07075054176967921</v>
+        <v>0.05890402007925618</v>
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>frozenset({'Iced Lychee Tea', 'Nasi Goreng Sambal Ijo'})</t>
+          <t>frozenset({'Americano Hot Bold', 'Americano Ice Bold'})</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>frozenset({'Iced Lychee Tea'})</t>
+          <t>frozenset({'Choco Berry'})</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>frozenset({'French Fries'})</t>
+          <t>frozenset({'Caramel Machiato'})</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>0.01749490179242245</v>
+        <v>0.02407577950269701</v>
       </c>
       <c r="D4" t="n">
-        <v>0.0264033487173983</v>
+        <v>0.07538481778713327</v>
       </c>
       <c r="E4" t="n">
-        <v>0.00157418339236521</v>
+        <v>0.002236547822654914</v>
       </c>
       <c r="F4" t="n">
-        <v>0.08997955010224948</v>
+        <v>0.09289617486338798</v>
       </c>
       <c r="G4" t="n">
-        <v>3.407884017490481</v>
+        <v>1.232292888545571</v>
       </c>
       <c r="H4" t="n">
         <v>1</v>
       </c>
       <c r="I4" t="n">
-        <v>0.001112259399563244</v>
+        <v>0.0004215995717609016</v>
       </c>
       <c r="J4" t="n">
-        <v>1.069862387589196</v>
+        <v>1.019304688825028</v>
       </c>
       <c r="K4" t="n">
-        <v>0.7191441396706854</v>
+        <v>0.1931549648708231</v>
       </c>
       <c r="L4" t="n">
-        <v>0.03719357565511412</v>
+        <v>0.02300405953991881</v>
       </c>
       <c r="M4" t="n">
-        <v>0.06530034927821171</v>
+        <v>0.01893907585893741</v>
       </c>
       <c r="N4" t="n">
-        <v>0.07480007315410576</v>
+        <v>0.06128229336537637</v>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>frozenset({'French Fries', 'Iced Lychee Tea'})</t>
+          <t>frozenset({'Caramel Machiato', 'Choco Berry'})</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>frozenset({'Lemon Tea Ice'})</t>
+          <t>frozenset({'Churros Beton'})</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>frozenset({'Tahu Goreng Lada Garam'})</t>
+          <t>frozenset({'Java Latte'})</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>0.01338055883510429</v>
+        <v>0.01144586238652809</v>
       </c>
       <c r="D5" t="n">
-        <v>0.02504382669671926</v>
+        <v>0.08985659781607683</v>
       </c>
       <c r="E5" t="n">
-        <v>0.001073306858430825</v>
+        <v>0.001249835547954217</v>
       </c>
       <c r="F5" t="n">
-        <v>0.0802139037433155</v>
+        <v>0.1091954022988506</v>
       </c>
       <c r="G5" t="n">
-        <v>3.202941176470588</v>
+        <v>1.215218525437135</v>
       </c>
       <c r="H5" t="n">
         <v>1</v>
       </c>
       <c r="I5" t="n">
-        <v>0.0007382064618592177</v>
+        <v>0.000221349294829801</v>
       </c>
       <c r="J5" t="n">
-        <v>1.059981420975078</v>
+        <v>1.02170936761292</v>
       </c>
       <c r="K5" t="n">
-        <v>0.6971147453796036</v>
+        <v>0.1791532998052759</v>
       </c>
       <c r="L5" t="n">
-        <v>0.02873563218390804</v>
+        <v>0.01249178172255096</v>
       </c>
       <c r="M5" t="n">
-        <v>0.05658723802904155</v>
+        <v>0.02124808512193745</v>
       </c>
       <c r="N5" t="n">
-        <v>0.06153552330022917</v>
+        <v>0.06155231315528181</v>
       </c>
       <c r="O5" t="inlineStr">
         <is>
-          <t>frozenset({'Lemon Tea Ice', 'Tahu Goreng Lada Garam'})</t>
+          <t>frozenset({'Java Latte', 'Churros Beton'})</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>frozenset({'Mineral Water'})</t>
+          <t>frozenset({'Spaghetti Aglio e Olio'})</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>frozenset({'Nasi Goreng Sambal Ijo'})</t>
+          <t>frozenset({'Caramel Machiato'})</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>0.06303888948517047</v>
+        <v>0.02190501249835548</v>
       </c>
       <c r="D6" t="n">
-        <v>0.02397051983828843</v>
+        <v>0.07538481778713327</v>
       </c>
       <c r="E6" t="n">
-        <v>0.004507888805409466</v>
+        <v>0.001973424549401395</v>
       </c>
       <c r="F6" t="n">
-        <v>0.07150964812712826</v>
+        <v>0.0900900900900901</v>
       </c>
       <c r="G6" t="n">
-        <v>2.983233096718451</v>
+        <v>1.195069414964703</v>
       </c>
       <c r="H6" t="n">
         <v>1</v>
       </c>
       <c r="I6" t="n">
-        <v>0.002996813854421515</v>
+        <v>0.00032211917358799</v>
       </c>
       <c r="J6" t="n">
-        <v>1.051200454795193</v>
+        <v>1.016161239857705</v>
       </c>
       <c r="K6" t="n">
-        <v>0.7095205972215403</v>
+        <v>0.1668841213262493</v>
       </c>
       <c r="L6" t="n">
-        <v>0.05464006938421509</v>
+        <v>0.02070393374741201</v>
       </c>
       <c r="M6" t="n">
-        <v>0.04870665205825894</v>
+        <v>0.01590420813528385</v>
       </c>
       <c r="N6" t="n">
-        <v>0.1297846748098328</v>
+        <v>0.05813405028064714</v>
       </c>
       <c r="O6" t="inlineStr">
         <is>
-          <t>frozenset({'Mineral Water', 'Nasi Goreng Sambal Ijo'})</t>
+          <t>frozenset({'Caramel Machiato', 'Spaghetti Aglio e Olio'})</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>frozenset({'Iced Lychee Tea'})</t>
+          <t>frozenset({'Earl Grey'})</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>frozenset({'Nasi Goreng Sambal Cikur'})</t>
+          <t>frozenset({'Java Latte'})</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>0.01749490179242245</v>
+        <v>0.009998684383633733</v>
       </c>
       <c r="D7" t="n">
-        <v>0.02085792994883904</v>
+        <v>0.08985659781607683</v>
       </c>
       <c r="E7" t="n">
-        <v>0.001073306858430825</v>
+        <v>0.001052493093014077</v>
       </c>
       <c r="F7" t="n">
-        <v>0.06134969325153374</v>
+        <v>0.1052631578947368</v>
       </c>
       <c r="G7" t="n">
-        <v>2.941312651927306</v>
+        <v>1.171457193496185</v>
       </c>
       <c r="H7" t="n">
         <v>1</v>
       </c>
       <c r="I7" t="n">
-        <v>0.0007083994223826592</v>
+        <v>0.0001540453316640128</v>
       </c>
       <c r="J7" t="n">
-        <v>1.043138283779995</v>
+        <v>1.017219096558502</v>
       </c>
       <c r="K7" t="n">
-        <v>0.6717682615978442</v>
+        <v>0.1478405315614618</v>
       </c>
       <c r="L7" t="n">
-        <v>0.02879078694817658</v>
+        <v>0.01065246338215712</v>
       </c>
       <c r="M7" t="n">
-        <v>0.04135432900005918</v>
+        <v>0.0169276182650903</v>
       </c>
       <c r="N7" t="n">
-        <v>0.0564038346189058</v>
+        <v>0.05848809432072127</v>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>frozenset({'Nasi Goreng Sambal Cikur', 'Iced Lychee Tea'})</t>
+          <t>frozenset({'Java Latte', 'Earl Grey'})</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>frozenset({'Lemon Tea Ice'})</t>
+          <t>frozenset({'Brownies with Ice Cream'})</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>frozenset({'French Fries'})</t>
+          <t>frozenset({'Java Latte'})</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>0.01338055883510429</v>
+        <v>0.01013024602026049</v>
       </c>
       <c r="D8" t="n">
-        <v>0.0264033487173983</v>
+        <v>0.08985659781607683</v>
       </c>
       <c r="E8" t="n">
-        <v>0.001037529963149798</v>
+        <v>0.001052493093014077</v>
       </c>
       <c r="F8" t="n">
-        <v>0.07754010695187166</v>
+        <v>0.1038961038961039</v>
       </c>
       <c r="G8" t="n">
-        <v>2.93675274988044</v>
+        <v>1.156243463710521</v>
       </c>
       <c r="H8" t="n">
         <v>1</v>
       </c>
       <c r="I8" t="n">
-        <v>0.0006842384021928745</v>
+        <v>0.0001422236505936173</v>
       </c>
       <c r="J8" t="n">
-        <v>1.055435210375922</v>
+        <v>1.0156672749009</v>
       </c>
       <c r="K8" t="n">
-        <v>0.6684318391263084</v>
+        <v>0.136513157894737</v>
       </c>
       <c r="L8" t="n">
-        <v>0.02677746999076639</v>
+        <v>0.01063829787234043</v>
       </c>
       <c r="M8" t="n">
-        <v>0.05252355599940341</v>
+        <v>0.01542559781935325</v>
       </c>
       <c r="N8" t="n">
-        <v>0.0584177499529006</v>
+        <v>0.05780456732140481</v>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>frozenset({'Lemon Tea Ice', 'French Fries'})</t>
+          <t>frozenset({'Java Latte', 'Brownies with Ice Cream'})</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>frozenset({'Mineral Water'})</t>
+          <t>frozenset({'Butter Croissant'})</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>frozenset({'Tahu Goreng Lada Garam'})</t>
+          <t>frozenset({'Java Latte'})</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>0.06303888948517047</v>
+        <v>0.02098408104196816</v>
       </c>
       <c r="D9" t="n">
-        <v>0.02504382669671926</v>
+        <v>0.08985659781607683</v>
       </c>
       <c r="E9" t="n">
-        <v>0.004615219491252549</v>
+        <v>0.002104986186028154</v>
       </c>
       <c r="F9" t="n">
-        <v>0.07321225879682181</v>
+        <v>0.1003134796238244</v>
       </c>
       <c r="G9" t="n">
-        <v>2.923365493757094</v>
+        <v>1.116372999444641</v>
       </c>
       <c r="H9" t="n">
         <v>1</v>
       </c>
       <c r="I9" t="n">
-        <v>0.003036484467832302</v>
+        <v>0.0002194280553000588</v>
       </c>
       <c r="J9" t="n">
-        <v>1.051973531757735</v>
+        <v>1.011622805911747</v>
       </c>
       <c r="K9" t="n">
-        <v>0.7021940390974257</v>
+        <v>0.1064763488543977</v>
       </c>
       <c r="L9" t="n">
-        <v>0.05529361337333905</v>
+        <v>0.01935874168179069</v>
       </c>
       <c r="M9" t="n">
-        <v>0.04940574091335974</v>
+        <v>0.01148926837535265</v>
       </c>
       <c r="N9" t="n">
-        <v>0.128748986541268</v>
+        <v>0.06186977055861793</v>
       </c>
       <c r="O9" t="inlineStr">
         <is>
-          <t>frozenset({'Tahu Goreng Lada Garam', 'Mineral Water'})</t>
+          <t>frozenset({'Butter Croissant', 'Java Latte'})</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>frozenset({'Mineral Water'})</t>
+          <t>frozenset({'Cookies Choco'})</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>frozenset({'French Fries'})</t>
+          <t>frozenset({'Java Latte'})</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>0.06303888948517047</v>
+        <v>0.02782528614655966</v>
       </c>
       <c r="D10" t="n">
-        <v>0.0264033487173983</v>
+        <v>0.08985659781607683</v>
       </c>
       <c r="E10" t="n">
-        <v>0.004686773281814604</v>
+        <v>0.002762794369161953</v>
       </c>
       <c r="F10" t="n">
-        <v>0.07434733257661748</v>
+        <v>0.09929078014184398</v>
       </c>
       <c r="G10" t="n">
-        <v>2.815829665107094</v>
+        <v>1.104991537127608</v>
       </c>
       <c r="H10" t="n">
         <v>1</v>
       </c>
       <c r="I10" t="n">
-        <v>0.003022335499980115</v>
+        <v>0.0002625088227732864</v>
       </c>
       <c r="J10" t="n">
-        <v>1.051794788203522</v>
+        <v>1.010474170928608</v>
       </c>
       <c r="K10" t="n">
-        <v>0.6882514918710408</v>
+        <v>0.09773520342571022</v>
       </c>
       <c r="L10" t="n">
-        <v>0.05529759392148586</v>
+        <v>0.02404121350887236</v>
       </c>
       <c r="M10" t="n">
-        <v>0.0492441955259999</v>
+        <v>0.01036559986385604</v>
       </c>
       <c r="N10" t="n">
-        <v>0.1259270538221841</v>
+        <v>0.06501874292597323</v>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>frozenset({'French Fries', 'Mineral Water'})</t>
+          <t>frozenset({'Java Latte', 'Cookies Choco'})</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>frozenset({'Iced Lychee Tea'})</t>
+          <t>frozenset({'Lemon Tea Ice'})</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>frozenset({'Tahu Goreng Lada Garam'})</t>
+          <t>frozenset({'Java Latte'})</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>0.01749490179242245</v>
+        <v>0.02453624523089067</v>
       </c>
       <c r="D11" t="n">
-        <v>0.02504382669671926</v>
+        <v>0.08985659781607683</v>
       </c>
       <c r="E11" t="n">
-        <v>0.001109083753711853</v>
+        <v>0.002302328640968294</v>
       </c>
       <c r="F11" t="n">
-        <v>0.06339468302658487</v>
+        <v>0.09383378016085792</v>
       </c>
       <c r="G11" t="n">
-        <v>2.531349693251534</v>
+        <v>1.044261439242578</v>
       </c>
       <c r="H11" t="n">
         <v>1</v>
       </c>
       <c r="I11" t="n">
-        <v>0.0006709444651463018</v>
+        <v>9.758512133951772e-05</v>
       </c>
       <c r="J11" t="n">
-        <v>1.040946656649136</v>
+        <v>1.004389020753264</v>
       </c>
       <c r="K11" t="n">
-        <v>0.6157258945498882</v>
+        <v>0.04345153800949896</v>
       </c>
       <c r="L11" t="n">
-        <v>0.02677029360967185</v>
+        <v>0.02053990610328639</v>
       </c>
       <c r="M11" t="n">
-        <v>0.03933597979068928</v>
+        <v>0.004369841428545974</v>
       </c>
       <c r="N11" t="n">
-        <v>0.05384019865614958</v>
+        <v>0.05972801745963833</v>
       </c>
       <c r="O11" t="inlineStr">
         <is>
-          <t>frozenset({'Tahu Goreng Lada Garam', 'Iced Lychee Tea'})</t>
+          <t>frozenset({'Java Latte', 'Lemon Tea Ice'})</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>frozenset({'Latte Ice Light'})</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>frozenset({'Java Latte'})</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>0.02236547822654914</v>
+      </c>
+      <c r="D12" t="n">
+        <v>0.08985659781607683</v>
+      </c>
+      <c r="E12" t="n">
+        <v>0.002039205367714775</v>
+      </c>
+      <c r="F12" t="n">
+        <v>0.0911764705882353</v>
+      </c>
+      <c r="G12" t="n">
+        <v>1.014688657307726</v>
+      </c>
+      <c r="H12" t="n">
+        <v>1</v>
+      </c>
+      <c r="I12" t="n">
+        <v>2.951958574752556e-05</v>
+      </c>
+      <c r="J12" t="n">
+        <v>1.001452287192666</v>
+      </c>
+      <c r="K12" t="n">
+        <v>0.0148071939260554</v>
+      </c>
+      <c r="L12" t="n">
+        <v>0.01850746268656717</v>
+      </c>
+      <c r="M12" t="n">
+        <v>0.001450181113208525</v>
+      </c>
+      <c r="N12" t="n">
+        <v>0.05693523382998881</v>
+      </c>
+      <c r="O12" t="inlineStr">
+        <is>
+          <t>frozenset({'Java Latte', 'Latte Ice Light'})</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>frozenset({'Cappucino Hot Light'})</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>frozenset({'Java Latte'})</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>0.01309038284436258</v>
+      </c>
+      <c r="D13" t="n">
+        <v>0.08985659781607683</v>
+      </c>
+      <c r="E13" t="n">
+        <v>0.001184054729640837</v>
+      </c>
+      <c r="F13" t="n">
+        <v>0.09045226130653267</v>
+      </c>
+      <c r="G13" t="n">
+        <v>1.006629045667577</v>
+      </c>
+      <c r="H13" t="n">
+        <v>1</v>
+      </c>
+      <c r="I13" t="n">
+        <v>7.797463136476144e-06</v>
+      </c>
+      <c r="J13" t="n">
+        <v>1.00065490074365</v>
+      </c>
+      <c r="K13" t="n">
+        <v>0.006672739526168835</v>
+      </c>
+      <c r="L13" t="n">
+        <v>0.01163542340012928</v>
+      </c>
+      <c r="M13" t="n">
+        <v>0.0006544721293661219</v>
+      </c>
+      <c r="N13" t="n">
+        <v>0.0518147104482883</v>
+      </c>
+      <c r="O13" t="inlineStr">
+        <is>
+          <t>frozenset({'Java Latte', 'Cappucino Hot Light'})</t>
         </is>
       </c>
     </row>

</xml_diff>